<commit_message>
Address PN model review feedback
</commit_message>
<xml_diff>
--- a/Examples/AcPowerSystem/PNSequenceControl_SingleBus＆4Bus/GflPN&GfmPN_4Bus.xlsx
+++ b/Examples/AcPowerSystem/PNSequenceControl_SingleBus＆4Bus/GflPN&GfmPN_4Bus.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Simplus-Grid-Tool-master-latest_version\Examples\AcPowerSystem\PNSequenceControl_SingleBus＆4Bus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B9BD96-11AE-47D7-BDE6-992D51292EF1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52988AB4-5100-4EAF-8C5E-960635B76148}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="19392" windowHeight="10392" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
   <si>
     <t>This sheet summarizes the parameters for power flow analysis</t>
   </si>
@@ -247,6 +247,10 @@
   </si>
   <si>
     <t>Xv</t>
+  </si>
+  <si>
+    <t>f_pll</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -255,7 +259,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="176" formatCode="0.00_ "/>
-    <numFmt numFmtId="181" formatCode="0.000"/>
+    <numFmt numFmtId="177" formatCode="0.000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -357,7 +361,7 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="11" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="181" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -898,7 +902,7 @@
         <v>21</v>
       </c>
       <c r="I2" t="s">
-        <v>22</v>
+        <v>74</v>
       </c>
       <c r="J2" t="s">
         <v>23</v>

</xml_diff>